<commit_message>
Jurisdiction-fair + recency scoring, metal filter, Quebec grades, Ontario drill
- implied grade credit for un-graded past producers (data-poor provinces compete)
- production RECENCY: pre-1980 workings earn ~nothing, recent producers prime
- known-worthless (iron/sulphur) + industrial commodities get no implied credit
  (Ecstall, marble quarries drop out); keyword-based industrial detection
- dominant-metal filter on priority page (by $/t) + Precious-only preset;
  expanded metal taxonomy (Li, V, REE, Sb, PGE, …)
- Quebec real grades w/ confidence tiers + production years from SIGEOM GPKG
- Ontario: real MDI drill intersections instead of 'N drill holes nearby'

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VazHKsFqB3DtVEsnETMYFv
</commit_message>
<xml_diff>
--- a/site/nt_leads.xlsx
+++ b/site/nt_leads.xlsx
@@ -618,7 +618,7 @@
         <v>325</v>
       </c>
       <c r="U2" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V2" t="n">
         <v>62.46251</v>
@@ -682,7 +682,7 @@
         <v>325</v>
       </c>
       <c r="U3" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V3" t="n">
         <v>62.47921</v>
@@ -746,7 +746,7 @@
         <v>325</v>
       </c>
       <c r="U4" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V4" t="n">
         <v>62.55281</v>
@@ -814,7 +814,7 @@
         <v>325</v>
       </c>
       <c r="U5" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V5" t="n">
         <v>62.55361</v>
@@ -878,7 +878,7 @@
         <v>325</v>
       </c>
       <c r="U6" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V6" t="n">
         <v>62.83331</v>
@@ -942,7 +942,7 @@
         <v>325</v>
       </c>
       <c r="U7" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V7" t="n">
         <v>62.84831</v>
@@ -1010,7 +1010,7 @@
         <v>325</v>
       </c>
       <c r="U8" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V8" t="n">
         <v>63.41941</v>
@@ -1074,7 +1074,7 @@
         <v>325</v>
       </c>
       <c r="U9" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V9" t="n">
         <v>63.85001</v>
@@ -1138,7 +1138,7 @@
         <v>325</v>
       </c>
       <c r="U10" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V10" t="n">
         <v>63.90001</v>
@@ -1202,7 +1202,7 @@
         <v>325</v>
       </c>
       <c r="U11" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V11" t="n">
         <v>63.96671</v>
@@ -1270,7 +1270,7 @@
         <v>325</v>
       </c>
       <c r="U12" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V12" t="n">
         <v>62.75001</v>
@@ -1334,7 +1334,7 @@
         <v>325</v>
       </c>
       <c r="U13" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V13" t="n">
         <v>63.69141</v>
@@ -1398,7 +1398,7 @@
         <v>325</v>
       </c>
       <c r="U14" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V14" t="n">
         <v>63.70831</v>
@@ -1462,7 +1462,7 @@
         <v>325</v>
       </c>
       <c r="U15" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V15" t="n">
         <v>63.76421</v>
@@ -1526,7 +1526,7 @@
         <v>325</v>
       </c>
       <c r="U16" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V16" t="n">
         <v>63.54581</v>
@@ -1590,7 +1590,7 @@
         <v>325</v>
       </c>
       <c r="U17" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V17" t="n">
         <v>63.13421</v>
@@ -1654,7 +1654,7 @@
         <v>325</v>
       </c>
       <c r="U18" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V18" t="n">
         <v>64.29722</v>
@@ -1718,7 +1718,7 @@
         <v>325</v>
       </c>
       <c r="U19" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V19" t="n">
         <v>64.50060999999999</v>
@@ -1786,7 +1786,7 @@
         <v>325</v>
       </c>
       <c r="U20" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V20" t="n">
         <v>64.33971</v>
@@ -1850,7 +1850,7 @@
         <v>325</v>
       </c>
       <c r="U21" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V21" t="n">
         <v>64.13611</v>
@@ -1914,7 +1914,7 @@
         <v>325</v>
       </c>
       <c r="U22" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V22" t="n">
         <v>64.12971</v>
@@ -1982,7 +1982,7 @@
         <v>325</v>
       </c>
       <c r="U23" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V23" t="n">
         <v>64.33920999999999</v>
@@ -2050,7 +2050,7 @@
         <v>325</v>
       </c>
       <c r="U24" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V24" t="n">
         <v>64.34721</v>
@@ -2114,7 +2114,7 @@
         <v>325</v>
       </c>
       <c r="U25" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V25" t="n">
         <v>64.07811</v>
@@ -2182,7 +2182,7 @@
         <v>325</v>
       </c>
       <c r="U26" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V26" t="n">
         <v>64.19831000000001</v>
@@ -2250,7 +2250,7 @@
         <v>325</v>
       </c>
       <c r="U27" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V27" t="n">
         <v>64.36830999999999</v>
@@ -2314,7 +2314,7 @@
         <v>325</v>
       </c>
       <c r="U28" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V28" t="n">
         <v>63.56222</v>
@@ -2382,7 +2382,7 @@
         <v>325</v>
       </c>
       <c r="U29" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V29" t="n">
         <v>63.06862</v>
@@ -2450,7 +2450,7 @@
         <v>325</v>
       </c>
       <c r="U30" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V30" t="n">
         <v>64.31782</v>
@@ -2514,7 +2514,7 @@
         <v>325</v>
       </c>
       <c r="U31" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V31" t="n">
         <v>64.81782</v>
@@ -2578,7 +2578,7 @@
         <v>325</v>
       </c>
       <c r="U32" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V32" t="n">
         <v>64.81062</v>
@@ -2642,7 +2642,7 @@
         <v>325</v>
       </c>
       <c r="U33" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V33" t="n">
         <v>64.77282</v>
@@ -2706,7 +2706,7 @@
         <v>325</v>
       </c>
       <c r="U34" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V34" t="n">
         <v>64.91782000000001</v>
@@ -2770,7 +2770,7 @@
         <v>325</v>
       </c>
       <c r="U35" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V35" t="n">
         <v>64.82142</v>
@@ -2834,7 +2834,7 @@
         <v>325</v>
       </c>
       <c r="U36" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V36" t="n">
         <v>64.83362</v>
@@ -2898,7 +2898,7 @@
         <v>325</v>
       </c>
       <c r="U37" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V37" t="n">
         <v>64.82501999999999</v>
@@ -2962,7 +2962,7 @@
         <v>325</v>
       </c>
       <c r="U38" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V38" t="n">
         <v>64.82892</v>
@@ -3026,7 +3026,7 @@
         <v>325</v>
       </c>
       <c r="U39" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V39" t="n">
         <v>64.78312</v>
@@ -3090,7 +3090,7 @@
         <v>325</v>
       </c>
       <c r="U40" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V40" t="n">
         <v>64.89172000000001</v>
@@ -3154,7 +3154,7 @@
         <v>325</v>
       </c>
       <c r="U41" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V41" t="n">
         <v>64.76562</v>
@@ -3218,7 +3218,7 @@
         <v>325</v>
       </c>
       <c r="U42" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V42" t="n">
         <v>64.75752</v>
@@ -3282,7 +3282,7 @@
         <v>325</v>
       </c>
       <c r="U43" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V43" t="n">
         <v>64.93442</v>
@@ -3346,7 +3346,7 @@
         <v>325</v>
       </c>
       <c r="U44" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V44" t="n">
         <v>64.91282</v>
@@ -3410,7 +3410,7 @@
         <v>325</v>
       </c>
       <c r="U45" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V45" t="n">
         <v>64.90942</v>
@@ -3474,7 +3474,7 @@
         <v>325</v>
       </c>
       <c r="U46" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V46" t="n">
         <v>64.88172</v>
@@ -3538,7 +3538,7 @@
         <v>325</v>
       </c>
       <c r="U47" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V47" t="n">
         <v>64.89282</v>
@@ -3602,7 +3602,7 @@
         <v>325</v>
       </c>
       <c r="U48" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V48" t="n">
         <v>64.93422</v>
@@ -3666,7 +3666,7 @@
         <v>325</v>
       </c>
       <c r="U49" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V49" t="n">
         <v>64.11812</v>
@@ -3730,7 +3730,7 @@
         <v>325</v>
       </c>
       <c r="U50" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V50" t="n">
         <v>64.17641999999999</v>
@@ -3798,7 +3798,7 @@
         <v>325</v>
       </c>
       <c r="U51" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V51" t="n">
         <v>64.71062000000001</v>
@@ -3862,7 +3862,7 @@
         <v>325</v>
       </c>
       <c r="U52" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V52" t="n">
         <v>64.66892</v>
@@ -3926,7 +3926,7 @@
         <v>325</v>
       </c>
       <c r="U53" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V53" t="n">
         <v>64.63392</v>
@@ -3990,7 +3990,7 @@
         <v>325</v>
       </c>
       <c r="U54" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V54" t="n">
         <v>64.58422</v>
@@ -4058,7 +4058,7 @@
         <v>325</v>
       </c>
       <c r="U55" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V55" t="n">
         <v>64.53612</v>
@@ -4122,7 +4122,7 @@
         <v>325</v>
       </c>
       <c r="U56" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V56" t="n">
         <v>64.53722</v>
@@ -4186,7 +4186,7 @@
         <v>325</v>
       </c>
       <c r="U57" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V57" t="n">
         <v>64.53502</v>
@@ -4250,7 +4250,7 @@
         <v>325</v>
       </c>
       <c r="U58" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V58" t="n">
         <v>64.82642</v>
@@ -4314,7 +4314,7 @@
         <v>300</v>
       </c>
       <c r="U59" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V59" t="n">
         <v>64.85581999999999</v>
@@ -4378,7 +4378,7 @@
         <v>325</v>
       </c>
       <c r="U60" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V60" t="n">
         <v>64.79532</v>
@@ -4442,7 +4442,7 @@
         <v>325</v>
       </c>
       <c r="U61" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V61" t="n">
         <v>64.78532</v>
@@ -4506,7 +4506,7 @@
         <v>325</v>
       </c>
       <c r="U62" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V62" t="n">
         <v>64.70562</v>
@@ -4570,7 +4570,7 @@
         <v>325</v>
       </c>
       <c r="U63" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V63" t="n">
         <v>64.72752</v>
@@ -4634,7 +4634,7 @@
         <v>325</v>
       </c>
       <c r="U64" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V64" t="n">
         <v>64.70392</v>
@@ -4698,7 +4698,7 @@
         <v>325</v>
       </c>
       <c r="U65" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V65" t="n">
         <v>64.30642</v>
@@ -4762,7 +4762,7 @@
         <v>325</v>
       </c>
       <c r="U66" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V66" t="n">
         <v>64.40812</v>
@@ -4826,7 +4826,7 @@
         <v>325</v>
       </c>
       <c r="U67" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V67" t="n">
         <v>64.45782</v>
@@ -4890,7 +4890,7 @@
         <v>325</v>
       </c>
       <c r="U68" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V68" t="n">
         <v>64.43671999999999</v>
@@ -4954,7 +4954,7 @@
         <v>325</v>
       </c>
       <c r="U69" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V69" t="n">
         <v>64.43222</v>
@@ -5022,7 +5022,7 @@
         <v>325</v>
       </c>
       <c r="U70" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V70" t="n">
         <v>64.43532</v>
@@ -5086,7 +5086,7 @@
         <v>325</v>
       </c>
       <c r="U71" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V71" t="n">
         <v>64.43612</v>
@@ -5150,7 +5150,7 @@
         <v>325</v>
       </c>
       <c r="U72" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V72" t="n">
         <v>64.44752</v>
@@ -5214,7 +5214,7 @@
         <v>325</v>
       </c>
       <c r="U73" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V73" t="n">
         <v>64.45222</v>
@@ -5278,7 +5278,7 @@
         <v>325</v>
       </c>
       <c r="U74" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V74" t="n">
         <v>64.43472</v>
@@ -5342,7 +5342,7 @@
         <v>325</v>
       </c>
       <c r="U75" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V75" t="n">
         <v>64.43062</v>
@@ -5406,7 +5406,7 @@
         <v>325</v>
       </c>
       <c r="U76" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V76" t="n">
         <v>64.44311999999999</v>
@@ -5470,7 +5470,7 @@
         <v>325</v>
       </c>
       <c r="U77" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V77" t="n">
         <v>63.02332</v>
@@ -5538,7 +5538,7 @@
         <v>325</v>
       </c>
       <c r="U78" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V78" t="n">
         <v>63.11222</v>
@@ -5606,7 +5606,7 @@
         <v>325</v>
       </c>
       <c r="U79" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V79" t="n">
         <v>63.99002</v>
@@ -5670,7 +5670,7 @@
         <v>325</v>
       </c>
       <c r="U80" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V80" t="n">
         <v>62.57281</v>
@@ -5738,7 +5738,7 @@
         <v>325</v>
       </c>
       <c r="U81" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V81" t="n">
         <v>65.57080999999999</v>
@@ -5802,7 +5802,7 @@
         <v>325</v>
       </c>
       <c r="U82" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V82" t="n">
         <v>65.46941</v>
@@ -5870,7 +5870,7 @@
         <v>325</v>
       </c>
       <c r="U83" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V83" t="n">
         <v>71.63831</v>
@@ -5938,7 +5938,7 @@
         <v>325</v>
       </c>
       <c r="U84" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V84" t="n">
         <v>71.54470999999999</v>
@@ -6006,7 +6006,7 @@
         <v>325</v>
       </c>
       <c r="U85" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V85" t="n">
         <v>71.52332</v>
@@ -6070,7 +6070,7 @@
         <v>325</v>
       </c>
       <c r="U86" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V86" t="n">
         <v>71.60032</v>
@@ -6138,7 +6138,7 @@
         <v>325</v>
       </c>
       <c r="U87" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V87" t="n">
         <v>71.69972</v>
@@ -6206,7 +6206,7 @@
         <v>325</v>
       </c>
       <c r="U88" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V88" t="n">
         <v>71.34611</v>
@@ -6274,7 +6274,7 @@
         <v>325</v>
       </c>
       <c r="U89" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V89" t="n">
         <v>71.43331000000001</v>
@@ -6342,7 +6342,7 @@
         <v>325</v>
       </c>
       <c r="U90" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V90" t="n">
         <v>71.32811</v>
@@ -6410,7 +6410,7 @@
         <v>325</v>
       </c>
       <c r="U91" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V91" t="n">
         <v>71.43331000000001</v>
@@ -6478,7 +6478,7 @@
         <v>325</v>
       </c>
       <c r="U92" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V92" t="n">
         <v>71.47971</v>
@@ -6546,7 +6546,7 @@
         <v>325</v>
       </c>
       <c r="U93" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V93" t="n">
         <v>71.50001</v>
@@ -6614,7 +6614,7 @@
         <v>325</v>
       </c>
       <c r="U94" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V94" t="n">
         <v>71.48311</v>
@@ -6682,7 +6682,7 @@
         <v>325</v>
       </c>
       <c r="U95" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V95" t="n">
         <v>71.03221000000001</v>
@@ -6746,7 +6746,7 @@
         <v>325</v>
       </c>
       <c r="U96" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V96" t="n">
         <v>71.03811</v>
@@ -6814,7 +6814,7 @@
         <v>325</v>
       </c>
       <c r="U97" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V97" t="n">
         <v>71.02141</v>
@@ -6878,7 +6878,7 @@
         <v>325</v>
       </c>
       <c r="U98" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V98" t="n">
         <v>71.04940999999999</v>
@@ -6942,7 +6942,7 @@
         <v>325</v>
       </c>
       <c r="U99" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V99" t="n">
         <v>71.08531000000001</v>
@@ -7006,7 +7006,7 @@
         <v>325</v>
       </c>
       <c r="U100" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V100" t="n">
         <v>71.11031</v>
@@ -7070,7 +7070,7 @@
         <v>325</v>
       </c>
       <c r="U101" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V101" t="n">
         <v>71.18311</v>
@@ -7134,7 +7134,7 @@
         <v>325</v>
       </c>
       <c r="U102" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V102" t="n">
         <v>71.19811</v>
@@ -7202,7 +7202,7 @@
         <v>325</v>
       </c>
       <c r="U103" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V103" t="n">
         <v>71.04940999999999</v>
@@ -7270,7 +7270,7 @@
         <v>325</v>
       </c>
       <c r="U104" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V104" t="n">
         <v>71.73562</v>
@@ -7338,7 +7338,7 @@
         <v>325</v>
       </c>
       <c r="U105" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V105" t="n">
         <v>71.43191</v>
@@ -7402,7 +7402,7 @@
         <v>325</v>
       </c>
       <c r="U106" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V106" t="n">
         <v>70.94190999999999</v>
@@ -7470,7 +7470,7 @@
         <v>325</v>
       </c>
       <c r="U107" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V107" t="n">
         <v>70.93720999999999</v>
@@ -7538,7 +7538,7 @@
         <v>325</v>
       </c>
       <c r="U108" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V108" t="n">
         <v>70.96611</v>
@@ -7606,7 +7606,7 @@
         <v>325</v>
       </c>
       <c r="U109" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V109" t="n">
         <v>71.63221</v>
@@ -7674,7 +7674,7 @@
         <v>325</v>
       </c>
       <c r="U110" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V110" t="n">
         <v>62.41611</v>
@@ -7742,7 +7742,7 @@
         <v>325</v>
       </c>
       <c r="U111" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V111" t="n">
         <v>62.49941</v>
@@ -7810,7 +7810,7 @@
         <v>325</v>
       </c>
       <c r="U112" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V112" t="n">
         <v>62.46611</v>
@@ -7878,7 +7878,7 @@
         <v>325</v>
       </c>
       <c r="U113" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V113" t="n">
         <v>62.93331</v>
@@ -7946,7 +7946,7 @@
         <v>325</v>
       </c>
       <c r="U114" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V114" t="n">
         <v>63.86391</v>
@@ -8010,7 +8010,7 @@
         <v>325</v>
       </c>
       <c r="U115" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V115" t="n">
         <v>64.88641</v>
@@ -8074,7 +8074,7 @@
         <v>325</v>
       </c>
       <c r="U116" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V116" t="n">
         <v>64.62281</v>
@@ -8142,7 +8142,7 @@
         <v>325</v>
       </c>
       <c r="U117" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V117" t="n">
         <v>64.93671000000001</v>
@@ -8210,7 +8210,7 @@
         <v>325</v>
       </c>
       <c r="U118" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V118" t="n">
         <v>64.40061</v>
@@ -8278,7 +8278,7 @@
         <v>325</v>
       </c>
       <c r="U119" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V119" t="n">
         <v>64.39331</v>
@@ -8346,7 +8346,7 @@
         <v>325</v>
       </c>
       <c r="U120" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V120" t="n">
         <v>64.39081</v>
@@ -8414,7 +8414,7 @@
         <v>325</v>
       </c>
       <c r="U121" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V121" t="n">
         <v>65.06061</v>
@@ -8478,7 +8478,7 @@
         <v>325</v>
       </c>
       <c r="U122" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V122" t="n">
         <v>64.94891</v>
@@ -8542,7 +8542,7 @@
         <v>325</v>
       </c>
       <c r="U123" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V123" t="n">
         <v>69.57890999999999</v>
@@ -8606,7 +8606,7 @@
         <v>325</v>
       </c>
       <c r="U124" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V124" t="n">
         <v>69.48721</v>
@@ -8670,7 +8670,7 @@
         <v>325</v>
       </c>
       <c r="U125" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V125" t="n">
         <v>69.46671000000001</v>
@@ -8734,7 +8734,7 @@
         <v>325</v>
       </c>
       <c r="U126" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="V126" t="n">
         <v>64.57171</v>
@@ -8802,7 +8802,7 @@
         <v>200</v>
       </c>
       <c r="U127" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="V127" t="n">
         <v>65.50001</v>
@@ -8870,7 +8870,7 @@
         <v>200</v>
       </c>
       <c r="U128" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="V128" t="n">
         <v>65.50001</v>

</xml_diff>